<commit_message>
Literatur matrisi tamamlandi (M01-M06)
</commit_message>
<xml_diff>
--- a/references/Literatur_Matrisi.xlsx
+++ b/references/Literatur_Matrisi.xlsx
@@ -46,7 +46,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F6FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -104,9 +99,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -796,30 +788,62 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>M05</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Liang, W., Yuksekgonul, M., Mao, Y., Wu, E., &amp; Zou, J. (2023). GPT detectors are biased against non-native English writers. Patterns, 4(7), 100779. doi:10.1016/j.patter.2023.100779</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Henüz okunmadı</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>GPT dedektörleri ana dili İngilizce olan ve olmayan yazarlara karşı adil davranıyor mu?</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Yedi yaygın GPT dedektörü; iki insan yazımı korpus: ABD 8. sınıf öğrenci kompozisyonları (ana dili İngilizce) ve TOEFL kompozisyonları (ana dili İngilizce olmayan). Ayrıca ICLR 2023'ten 1.574 kabul edilmiş makale özeti.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Aynı dedektörlerin iki korpus üzerinde çalıştırılıp yanlış pozitif oranlarının karşılaştırılması; perplexity analizi; sözcük çeşitliliğini artıran müdahaleyle yeniden test</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Yanlış pozitif oranı (gruplara göre); metin perplexity değeri; müdahale sonrası değişim</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Dedektörler ana dili İngilizce olmayan yazarların metinlerini sistematik olarak YZ üretimi diye işaretliyor: TOEFL kompozisyonlarının yarısından fazlası yanlış sınıflandırılırken ana dili İngilizce olanların metinlerinde doğruluk neredeyse kusursuz. Mekanizma perplexity: sınırlı sözcük ve dilbilgisi çeşitliliği düşük perplexity üretiyor, dedektörler düşük perplexity'yi YZ işareti sayıyor. Sözcük çeşitliliğini artıran basit bir müdahale hem önyargıyı kaldırıyor hem de dedektörleri atlatıyor.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>İngilizce yazan, ana dili İngilizce olmayan yazarlara odaklanıyor; Türkçe yazılmış Türkçe metinleri kapsamıyor; dedektör sürümleri zamana bağlı</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>H4 hipotezinin teorik omurgası: Türkçe yazan bir kişi, İngilizce merkezli bir dedektör açısından tam da bu "non-native" konumunda. H2 ile de bağlantılı: düşük perplexity → yanlış pozitif zinciri, kısa ve kalıplaşmış cevapların neden daha riskli olabileceğini açıklıyor; length_band değişkenimizin gerekçesi buradan geliyor. Ayrıca projenin adalet/etik gerekçesini veriyor: dedektör hatası nötr değil, belirli grupları sistematik olarak etkiliyor.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Dâhil — temel kaynak</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Hem gerekçeyi (adalet) hem mekanizmayı (perplexity) veriyor. H1 (eğitim seviyesi ekseni) ile birlikte okunmalı: perplexity dilsel çeşitlilikle ilişkiliyse, ünvan arttıkça yanlış pozitifin düşmesi beklenebilir.</t>
         </is>
       </c>
     </row>
@@ -837,50 +861,82 @@
       <c r="C7" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Ayrı bir sınıflandırıcı eğitmeden, veri toplamadan ve filigran kullanmadan, yalnızca modelin olasılık yapısından yararlanarak YZ metni tespit edilebilir mi?</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Farklı üretim senaryoları; 20 milyar parametreli GPT-NeoX ile üretilmiş sahte haber metinleri dâhil çeşitli değerlendirme kümeleri</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Sıfır-atış (zero-shot) tespit: metnin, ilgilenilen modelin log-olasılık fonksiyonunda negatif eğrilik bölgesinde yer alma eğiliminden yararlanan eğrilik temelli ölçüt. Metne başka bir genel amaçlı dil modeliyle (ör. T5) rastgele bozulmalar uygulanıp log-olasılık değişimi ölçülüyor.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Log-olasılık; eğrilik (curvature) ölçütü; AUROC</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>YZ metinleri modelin log-olasılık fonksiyonunda negatif eğrilik bölgelerini işgal etme eğiliminde. Bu gözleme dayanan DetectGPT mevcut sıfır-atış yöntemlerinden daha ayırt edici: GPT-NeoX ile üretilmiş sahte haberlerde en güçlü sıfır-atış temelini 0,81 AUROC'tan 0,95 AUROC'a çıkarıyor. Yöntem sınıflandırıcı eğitimi, veri seti toplama veya filigran gerektirmiyor.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Kaynak modelin log-olasılıklarına erişim gerektiriyor (beyaz kutu varsayımı); metni hangi modelin ürettiği bilinmediğinde doğrudan uygulanamaz. Türkçe değerlendirilmemiş. M04'te DIPPER parafrazı karşısında başarımının %4,6'ya düştüğü gösterilmiş. Hesaplama maliyeti yüksek.</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Projedeki "temel model" (baseline) adayı: KARDEP Bölüm 11'deki açık kaynak/perplexity tabanlı tekrarlanabilir referans tam olarak bu tür bir yöntem. ANCAK kaynak modele erişim gereksinimi bizim denetim senaryomuzda sorun yaratıyor — metni hangi modelin yazdığını bilmiyoruz, dedektöre zaten bunu soruyoruz. Uyarlanmış (vekil model kullanan) veya daha basit bir perplexity temelli baseline gerekebilir. Danışmanla görüşülecek.</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Dâhil — temel kaynak</t>
+        </is>
+      </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Henüz okunmadı</t>
+          <t>M04 ile birlikte okunmalı: DetectGPT hem baseline adayımız hem de parafraz karşısında en net çöken dedektör (%70,3 → %4,6). Bu ikisi projenin evasion ekseninin iki ucu.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>AÇIKLAMA:</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>M01–M04: Okunmuş ve doldurulmuş kayıtlar. M05–M06: Sarı hücreler okundukça doldurulacak.</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>M01–M06: KARDEP proje metninin kaynakça bölümündeki altı temel makale (14–17.07.2026 tarihleri arasında okundu).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Kural (Usul-Esaslar 2.6): Hücreler makale özetinden kopyalanmaz; amaç, yöntem ve bulgu kendi cümlelerinle yazılır.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Yeni makale ekledikçe alta satır aç ve ID'yi sırayla ver (M07, M08, ...).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Dosya tek sürüm olarak yaşar; _v2 gibi kopya açma (Usul-Esaslar 5.3). Sürüm geçmişi Git'te tutulur.</t>
         </is>

</xml_diff>